<commit_message>
Rewrite verification-case init.xlsx files as Windows Excel exports.
Loaded roundtrip/default/scratch inits were Mac Excel, Excel Online, Openpyxl, POI 12/14, and other third-party ZIPs. Open each unique init in Excel and Save As xlsx format 51, then replace the file. Byte-identical inits are exported once and copied.

Add CheckWindowsExcel16Export and a corpus test that every loaded init has Application "Microsoft Excel" and AppVersion 16.x. Internal rewrite CLI: go run ./internal/excel-export-inits [cases-dir].
</commit_message>
<xml_diff>
--- a/verification/cases/default/add_sheet_sparse_ids/init.xlsx
+++ b/verification/cases/default/add_sheet_sparse_ids/init.xlsx
@@ -1,16 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frl\AppData\Local\Temp\xlsx-export-inits-1516826600\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCBD7446-C644-4D4F-8152-D01A3BD68F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Imported" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB7}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB7}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -18,7 +25,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -54,6 +61,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -373,13 +390,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rewrite verification-case init.xlsx files as Windows Excel exports (#32)
* Rewrite verification-case init.xlsx files as Windows Excel exports.

Loaded roundtrip/default/scratch inits were Mac Excel, Excel Online, Openpyxl, POI 12/14, and other third-party ZIPs. Open each unique init in Excel and Save As xlsx format 51, then replace the file. Byte-identical inits are exported once and copied.

Add CheckWindowsExcel16Export and a corpus test that every loaded init has Application "Microsoft Excel" and AppVersion 16.x. Internal rewrite CLI: go run ./internal/excel-export-inits [cases-dir].

* Expect roundtrip/formulas init to match its golden after Excel Save As.

The corpus test required stale cached v=0 vs golden 15. Rewriting inits as Windows Excel exports fills those caches, so CompareFiles is now equal. Cached 0 vs 15 stays covered by TestCompareUnequalOnCachedFormulaValue.
</commit_message>
<xml_diff>
--- a/verification/cases/default/add_sheet_sparse_ids/init.xlsx
+++ b/verification/cases/default/add_sheet_sparse_ids/init.xlsx
@@ -1,16 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frl\AppData\Local\Temp\xlsx-export-inits-1516826600\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BCBD7446-C644-4D4F-8152-D01A3BD68F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Imported" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB7}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB7}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -18,7 +25,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -54,6 +61,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -373,13 +390,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>